<commit_message>
Update the feature plan
Mark the work finished since the last plan refresh: enemy AI, waves, HUD,
model loading, skybox, terrain, score, game state and script properties.
Script hot-reload becomes Partial - the Inspector reloads on demand, but
nothing watches the file on disk.

Physics is no longer one optional row. M6 becomes seven phases: collider
shapes, Jolt integration, a forces API, the flight model as forces,
collision damage with raycast bullets, a terrain heightfield collider and
compound colliders. Adds the two missing rows for directional lighting and
for the data-flow visual scripting language.
</commit_message>
<xml_diff>
--- a/jetgame_plan.xlsx
+++ b/jetgame_plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ali_g\Documents\Staj\projects\imguiraylib-game\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF089308-A5FE-4996-B75D-9FD0F48000C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70296B9A-6FED-4313-9069-CFDD53626134}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1515" yWindow="1515" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="122">
   <si>
     <t>#</t>
   </si>
@@ -303,9 +303,6 @@
     <t>Script hot-reload</t>
   </si>
   <si>
-    <t>Tweak flight/AI scripts live without a rebuild - big dev-speed win.</t>
-  </si>
-  <si>
     <t>Game state (menu / play / win / lose / restart)</t>
   </si>
   <si>
@@ -327,16 +324,73 @@
     <t>Start screen, restart and settings - the shell around the loop.</t>
   </si>
   <si>
-    <t>O1</t>
-  </si>
-  <si>
-    <t>Rigid-body physics (collision response)</t>
-  </si>
-  <si>
     <t>M6 Physics</t>
   </si>
   <si>
-    <t>Bodies that collide and bounce: enables knockback, tumbling debris, gravity-arced projectiles. Not required for the core game - the flight model already gives realistic flying.</t>
+    <t>Partial</t>
+  </si>
+  <si>
+    <t>Tweak flight/AI scripts live without a rebuild - big dev-speed win. Partial: the Inspector has a manual Reload button; there is no automatic reload when the file changes on disk.</t>
+  </si>
+  <si>
+    <t>Collider shapes (Sphere / Box / Capsule)</t>
+  </si>
+  <si>
+    <t>Collision volumes with a local offset and rotation, sized in the Inspector. Replaces the sphere-only hitbox and is the per-body shape a physics engine needs.</t>
+  </si>
+  <si>
+    <t>Jolt integration (PhysicsWorld + RigidBody)</t>
+  </si>
+  <si>
+    <t>Adds the Jolt library, one physics body per Collider+RigidBody, stepped each frame with transforms synced back. Dynamic mode: physics moves the bodies, scripts no longer set positions directly.</t>
+  </si>
+  <si>
+    <t>Forces API for Lua (force / torque / impulse / velocity)</t>
+  </si>
+  <si>
+    <t>Scripts push bodies instead of teleporting them - the only way gameplay can drive dynamic physics.</t>
+  </si>
+  <si>
+    <t>Flight model rewritten as forces</t>
+  </si>
+  <si>
+    <t>Thrust, lift and drag become real forces on the jet body. The hardest step: prototype early, because it decides whether flying still feels right.</t>
+  </si>
+  <si>
+    <t>Collision damage + raycast bullets</t>
+  </si>
+  <si>
+    <t>A contact listener turns real collisions into damage, and bullets become raycasts so a fast shot cannot pass through a target between two frames. Retires the distance-based hit test.</t>
+  </si>
+  <si>
+    <t>Terrain heightfield collider (ground / crash)</t>
+  </si>
+  <si>
+    <t>Makes the ground solid, so flying into it crashes instead of passing through.</t>
+  </si>
+  <si>
+    <t>27, 19</t>
+  </si>
+  <si>
+    <t>Compound colliders + parented body sync</t>
+  </si>
+  <si>
+    <t>Several colliders under one body, for shapes a single primitive cannot cover, plus a world-to-local bridge so a parented dynamic body behaves.</t>
+  </si>
+  <si>
+    <t>Directional lighting + shading</t>
+  </si>
+  <si>
+    <t>Terrain and models currently render flat and unlit; one directional light plus a shader gives them form and depth.</t>
+  </si>
+  <si>
+    <t>F8</t>
+  </si>
+  <si>
+    <t>Data-flow visual scripting (typed pins, variables, codegen)</t>
+  </si>
+  <si>
+    <t>A full Blueprints-style node language that generates Lua: typed pins, variables, params, branches and loops. Grew out of F7; every gameplay script has been reproduced as a graph.</t>
   </si>
 </sst>
 </file>
@@ -389,12 +443,6 @@
   </cellStyles>
   <dxfs count="10">
     <dxf>
-      <alignment vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -418,6 +466,12 @@
     <dxf>
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -432,17 +486,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7F35B493-CEB0-4271-8DAD-91FE98C15FB8}" name="Table1" displayName="Table1" ref="A5:H39" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
-  <autoFilter ref="A5:H39" xr:uid="{7F35B493-CEB0-4271-8DAD-91FE98C15FB8}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7F35B493-CEB0-4271-8DAD-91FE98C15FB8}" name="Table1" displayName="Table1" ref="A5:H47" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+  <autoFilter ref="A5:H47" xr:uid="{7F35B493-CEB0-4271-8DAD-91FE98C15FB8}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{7E36C9AB-E4E2-4F80-9B0B-CF7219223D7D}" name="#" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{BE048A2A-36A1-4BF3-8DF0-9604E1A2C153}" name="Feature" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{AF6114BD-D77A-468D-AD11-36EB7D4E077C}" name="Milestone" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{256B4F5D-1201-4C5B-B0E8-AD8ACD331FD4}" name="Side" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{43F06B1D-F4D3-4947-9245-F3F00BACCD5C}" name="Priority" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{F35E2158-4E4B-455C-B865-A668E2F74031}" name="Status" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{643537F0-4CDF-4558-A3A1-E97E0339902F}" name="Why we need it" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{A0F9D607-5B28-42BA-98CF-29B15AC007F2}" name="Depends on" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{7E36C9AB-E4E2-4F80-9B0B-CF7219223D7D}" name="#" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{BE048A2A-36A1-4BF3-8DF0-9604E1A2C153}" name="Feature" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{AF6114BD-D77A-468D-AD11-36EB7D4E077C}" name="Milestone" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{256B4F5D-1201-4C5B-B0E8-AD8ACD331FD4}" name="Side" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{43F06B1D-F4D3-4947-9245-F3F00BACCD5C}" name="Priority" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{F35E2158-4E4B-455C-B865-A668E2F74031}" name="Status" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{643537F0-4CDF-4558-A3A1-E97E0339902F}" name="Why we need it" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{A0F9D607-5B28-42BA-98CF-29B15AC007F2}" name="Depends on" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight13" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -711,7 +765,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A5:H39"/>
+  <dimension ref="A5:H47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.5703125" style="2" bestFit="1" customWidth="1"/>
@@ -1262,7 +1316,7 @@
         <v>49</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="G25" s="3" t="s">
         <v>68</v>
@@ -1288,7 +1342,7 @@
         <v>36</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="G26" s="3" t="s">
         <v>71</v>
@@ -1314,7 +1368,7 @@
         <v>49</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="G27" s="3" t="s">
         <v>74</v>
@@ -1366,7 +1420,7 @@
         <v>36</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="G29" s="3" t="s">
         <v>79</v>
@@ -1392,7 +1446,7 @@
         <v>49</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="G30" s="3" t="s">
         <v>81</v>
@@ -1418,7 +1472,7 @@
         <v>49</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="G31" s="3" t="s">
         <v>83</v>
@@ -1444,7 +1498,7 @@
         <v>49</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="G32" s="3" t="s">
         <v>85</v>
@@ -1522,10 +1576,10 @@
         <v>49</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>54</v>
+        <v>100</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="H35" s="2" t="s">
         <v>22</v>
@@ -1536,10 +1590,10 @@
         <v>23</v>
       </c>
       <c r="B36" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="C36" s="3" t="s">
         <v>93</v>
-      </c>
-      <c r="C36" s="3" t="s">
-        <v>94</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>39</v>
@@ -1548,10 +1602,10 @@
         <v>36</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H36" s="2">
         <v>11</v>
@@ -1562,10 +1616,10 @@
         <v>24</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>44</v>
@@ -1574,10 +1628,10 @@
         <v>49</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="H37" s="2">
         <v>23</v>
@@ -1588,10 +1642,10 @@
         <v>25</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>11</v>
@@ -1603,36 +1657,244 @@
         <v>54</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="H38" s="2">
         <v>23</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="2" t="s">
-        <v>100</v>
+      <c r="A39" s="2">
+        <v>26</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>87</v>
+        <v>36</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="G39" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="H39" s="2" t="s">
-        <v>15</v>
+      <c r="H39" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="A40" s="2">
+        <v>27</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="G40" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="H40" s="2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A41" s="2">
+        <v>28</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="G41" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="H41" s="2">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A42" s="2">
+        <v>29</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="G42" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="H42" s="2">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="A43" s="2">
+        <v>30</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="G43" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="H43" s="2">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A44" s="2">
+        <v>31</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="G44" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A45" s="2">
+        <v>32</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="G45" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="H45" s="2">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A46" s="2">
+        <v>33</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="G46" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="H46" s="2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="A47" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G47" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="H47" s="2" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bring the plan up to date with the branch
Eight statuses were stale: Jolt, the forces API, collision damage and the
terrain collider are all done, ground vehicles landed with the camps, and
audio is no longer partial now every sound has a file. Compound colliders
drop to partial - the parented-body half is done, the compound half is
not.

Two rows would have been misleading marked Done, so their descriptions
say what actually happened: the flight model was never rewritten as
forces (JSBSim owns the state instead, exactly as the roadmap predicted),
and bullets became swept dynamic bodies rather than raycasts.

Four new rows for the JSBSim work: the flight model, the terrain feeding
it, the exhaust plume and fuel.
</commit_message>
<xml_diff>
--- a/jetgame_plan.xlsx
+++ b/jetgame_plan.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="132">
   <si>
     <t>#</t>
   </si>
@@ -391,6 +391,36 @@
   </si>
   <si>
     <t>A huge feel multiplier; raylib has audio built in. Engine side done: sounds are defined as data in assets/scripts/sounds.lua, with voice pooling for overlap, per-play pitch variation, and a throttle-driven engine loop. Partial only because no sound FILES exist yet - each one is registered and silent until a file is dropped into assets/sounds/.</t>
+  </si>
+  <si>
+    <t>JSBSim flight dynamics model (real aerodynamics)</t>
+  </si>
+  <si>
+    <t>A full aerodynamic simulation of a named aircraft, read from XML at runtime: lift and drag curves, engine thrust, mass and inertia. Quarantined inside FlightModel.cpp the way Jolt is inside Physics.cpp. The jet stalls, bleeds speed in a turn and mushes when slow, none of it written anywhere.</t>
+  </si>
+  <si>
+    <t>Terrain fed to the flight model (ground strikes)</t>
+  </si>
+  <si>
+    <t>A KINEMATIC body never collides with STATIC terrain whatever it is set to - measured, a capsule fell 2000 m through a 440 m hill with no contact - so ground impact cannot come from the physics engine. The flight model is told the ground height beneath the aircraft each frame and reports the strike through the normal onCollision hook.</t>
+  </si>
+  <si>
+    <t>Engine exhaust + afterburner plume</t>
+  </si>
+  <si>
+    <t>Visible thrust: a dry shimmer and a reheat flame from the tailpipe. Driven by the ENGINE throttle position rather than the lever, so the burner lights where the aircraft really lights it - half throttle on the F-16, whose control system doubles the lever onto the engine 0-to-2 range.</t>
+  </si>
+  <si>
+    <t>Fuel: HUD gauge, low-fuel warning, start load</t>
+  </si>
+  <si>
+    <t>Fuel is finite in the model and running dry looks exactly like a bug - the throttle stops doing anything. A gauge and a flashing caption, an unlimited-fuel option (on by default) and a per-aircraft start load in the Inspector.</t>
+  </si>
+  <si>
+    <t>SUPERSEDED BY JSBSIM. The flight model was never rewritten as forces: JSBSim integrates its own state and fights being pushed, exactly as the roadmap predicted, so it OWNS the aircraft position and writes the transform. The rigid body stays Kinematic and Jolt does collision only.</t>
+  </si>
+  <si>
+    <t>A contact listener turns real collisions into damage. Bullets became dynamic bodies with CONTINUOUS collision rather than raycasts - a swept path solves the same tunnelling problem and brings bullet drop, ground and scenery hits for free. Retires the distance-based hit test.</t>
   </si>
 </sst>
 </file>
@@ -486,8 +516,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7F35B493-CEB0-4271-8DAD-91FE98C15FB8}" name="Table1" displayName="Table1" ref="A5:H47" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
-  <autoFilter ref="A5:H47" xr:uid="{7F35B493-CEB0-4271-8DAD-91FE98C15FB8}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7F35B493-CEB0-4271-8DAD-91FE98C15FB8}" name="Table1" displayName="Table1" ref="A5:H51" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+  <autoFilter ref="A5:H51" xr:uid="{7F35B493-CEB0-4271-8DAD-91FE98C15FB8}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{7E36C9AB-E4E2-4F80-9B0B-CF7219223D7D}" name="#" dataDxfId="7"/>
     <tableColumn id="2" xr3:uid="{BE048A2A-36A1-4BF3-8DF0-9604E1A2C153}" name="Feature" dataDxfId="6"/>
@@ -765,7 +795,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A5:H47"/>
+  <dimension ref="A5:H51"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.5703125" style="2" bestFit="1" customWidth="1"/>
@@ -1394,7 +1424,7 @@
         <v>49</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="G28" s="3" t="s">
         <v>76</v>
@@ -1550,7 +1580,7 @@
         <v>49</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>99</v>
+        <v>12</v>
       </c>
       <c r="G34" s="3" t="s">
         <v>121</v>
@@ -1706,7 +1736,7 @@
         <v>36</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="G40" s="3" t="s">
         <v>104</v>
@@ -1732,7 +1762,7 @@
         <v>36</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="G41" s="3" t="s">
         <v>106</v>
@@ -1758,10 +1788,10 @@
         <v>36</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>108</v>
+        <v>130</v>
       </c>
       <c r="H42" s="2">
         <v>28</v>
@@ -1784,10 +1814,10 @@
         <v>36</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>110</v>
+        <v>131</v>
       </c>
       <c r="H43" s="2">
         <v>27</v>
@@ -1810,7 +1840,7 @@
         <v>49</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="G44" s="3" t="s">
         <v>112</v>
@@ -1836,7 +1866,7 @@
         <v>49</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>54</v>
+        <v>99</v>
       </c>
       <c r="G45" s="3" t="s">
         <v>115</v>
@@ -1895,6 +1925,110 @@
       </c>
       <c r="H47" s="2" t="s">
         <v>31</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="A48" s="2">
+        <v>34</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G48" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="H48" s="2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="A49" s="2">
+        <v>35</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G49" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="H49" s="2">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="A50" s="2">
+        <v>36</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G50" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="H50" s="2">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="A51" s="2">
+        <v>37</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G51" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="H51" s="2">
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>